<commit_message>
Add invoice numbers per HS code to Donaldson Kadan summary
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VYoChnHAkutVKnEY4irnRy
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Donaldson_Kadan_DON_WUXI_2026_05_12.xlsx
+++ b/output/HS_Code_Summary_Donaldson_Kadan_DON_WUXI_2026_05_12.xlsx
@@ -65,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -80,6 +80,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -446,18 +449,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,32 +480,37 @@
           <t>Země původu (COO)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Faktura (č.)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Celkové množství (ks)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hodnota CNY</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Příznak</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>TARIC / poznámka / CBAM / Antidumping</t>
         </is>
@@ -523,20 +532,24 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>30600162208, 30600162209</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>20</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>850</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>1400</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>166558.24</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -554,20 +567,24 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>30600162209, 30600162250</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>570</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>760</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>49942.37</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -585,20 +602,24 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>30600162210</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>4</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>52</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>80</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>6971.69</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -616,20 +637,24 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>30600162209</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>6</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>33</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>85</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>5035.32</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -647,24 +672,29 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>30600162250</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="F6" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="G6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="H6" s="3" t="n">
         <v>374.63</v>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>CBAM zboží (železo/ocel, kap. 73). Čistá hmotnost 0,5 kg – de minimis → kód Y137 v JSD. AD clo na spojovací materiál z CN (nař. 2022/191) se na 7318 23 (nýty) NEvztahuje – pokrývá jen 7318 12/14/15/21/22.</t>
         </is>
@@ -686,24 +716,29 @@
           <t>CN</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>30600162250</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="F7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="G7" s="3" t="n">
         <v>1.5</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="H7" s="3" t="n">
         <v>284.96</v>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>CBAM zboží (železo/ocel, kap. 73). Čistá hmotnost pouze 1 kg – hluboko pod limitem de minimis 50 t/rok → kód Y137 v JSD (potvrdit se zákazníkem). Pozor: AD clo na potrubní tvarovky z CN (ex 7307 99 80, 58,6 %) – ověřit v TARIC, zda se na díl vztahuje (pravděpodobně ne, není svařovací tvarovka).</t>
         </is>
@@ -717,21 +752,23 @@
       </c>
       <c r="B8" s="6" t="inlineStr"/>
       <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="F8" s="5" t="n">
         <v>1506.5</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="G8" s="5" t="n">
         <v>2327.5</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="H8" s="5" t="n">
         <v>229167.21</v>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
-    </row>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -840,9 +877,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="5">
         <f>== PŘIJATÉ DOKUMENTY (stav 10.7.2026) ===</f>
@@ -884,9 +919,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="5">
         <f>== PREFERENČNÍ VĚTA / COO – DŮLEŽITÉ ===</f>
@@ -914,9 +947,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5">
         <f>== CBAM ===</f>
@@ -944,9 +975,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="5">
         <f>== ANTIDUMPING ===</f>
@@ -974,9 +1003,7 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="5">
         <f>== POZNÁMKY / NESROVNALOSTI ===</f>

</xml_diff>

<commit_message>
Merge air filtration items under EU TARIC 8421392590 (CN export codes 8421392990/8421392290 do not exist in EU tariff)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VYoChnHAkutVKnEY4irnRy
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Donaldson_Kadan_DON_WUXI_2026_05_12.xlsx
+++ b/output/HS_Code_Summary_Donaldson_Kadan_DON_WUXI_2026_05_12.xlsx
@@ -30,7 +30,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -83,6 +88,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,13 +458,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -467,7 +476,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HS kód</t>
+          <t>HS kód (EU TARIC)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -480,7 +489,7 @@
           <t>Země původu (COO)</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Faktura (č.)</t>
         </is>
@@ -519,12 +528,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8421392990</t>
+          <t>8421392590</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Sběrače prachu</t>
+          <t>Stroje a přístroje pro filtrování nebo čištění vzduchu – sběrače prachu (DCE125) a předvyrobené filtrační jednotky (UMA)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -534,137 +543,169 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>30600162208, 30600162209</t>
+          <t>30600162208, 30600162209, 30600162250</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F2" t="n">
-        <v>850</v>
+        <v>1420</v>
       </c>
       <c r="G2" t="n">
-        <v>1400</v>
+        <v>2160</v>
       </c>
       <c r="H2" t="n">
-        <v>166558.24</v>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
+        <v>216500.61</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>EU kód 8421 39 25 90 (ostatní, ne pro civilní letadla). Sloučeno z čínských exportních kódů 8421392990 + 8421392290 – v TARIC EU neexistují, oba spadají pod filtraci vzduchu.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>8421392290</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Vrchní a spodní část předvyrobené filtrační jednotky (UMA)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>8421199090</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Sada pro uzemnění sběrné nádoby filtru (BIN BASE PACK)</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>30600162209, 30600162250</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>570</v>
-      </c>
-      <c r="G3" t="n">
-        <v>760</v>
-      </c>
-      <c r="H3" t="n">
-        <v>49942.37</v>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>30600162210</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>6971.69</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Čínský exportní kód. EU členění 8421 19 je jiné (8421 19 20 laboratorní / 8421 19 70 ostatní odstředivky) – ověřit správné EU zařazení, položka možná patří spíše do částí 8421 99.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>8421199090</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Sada pro uzemnění sběrné nádoby filtru</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>8421999090</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Sběrná nádoba filtru (dust bins)</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>30600162210</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>30600162209</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>85</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>5035.32</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>OVĚŘIT</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Čínský exportní kód. V EU CN odpovídá 8421 99 90 (ostatní části a součásti) – ověřit přesný TARIC při podání JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>7318230000</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Sada pro upevnění těsnícího zařízení (nýty)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>30600162250</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F4" t="n">
-        <v>52</v>
-      </c>
-      <c r="G4" t="n">
-        <v>80</v>
-      </c>
-      <c r="H4" t="n">
-        <v>6971.69</v>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>8421999090</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Sběrná nádoba filtru</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>30600162209</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" t="n">
-        <v>33</v>
-      </c>
-      <c r="G5" t="n">
-        <v>85</v>
-      </c>
-      <c r="H5" t="n">
-        <v>5035.32</v>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="F5" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>374.63</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>EU kód 7318 23 00 existuje shodně. CBAM zboží (železo/ocel, kap. 73), NW 0,5 kg – de minimis → kód Y137 v JSD. AD clo na spojovací materiál z CN (nař. 2022/191) se na 7318 23 NEvztahuje.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>7318230000</t>
+          <t>7307990000</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Sada pro upevnění těsnícího zařízení</t>
+          <t>Sestava vyrovnávacího kohoutu zásobníku na prach</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -681,13 +722,13 @@
         <v>4</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>374.63</v>
+        <v>284.96</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
@@ -696,119 +737,98 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>CBAM zboží (železo/ocel, kap. 73). Čistá hmotnost 0,5 kg – de minimis → kód Y137 v JSD. AD clo na spojovací materiál z CN (nař. 2022/191) se na 7318 23 (nýty) NEvztahuje – pokrývá jen 7318 12/14/15/21/22.</t>
+          <t>Čínský kód; EU ekvivalent 7307 99 80 (ostatní příslušenství pro trouby/trubky). CBAM zboží, NW 1 kg – de minimis → Y137. AD clo na svařovací tvarovky z CN (ex 7307 99 80, 58,6 %) – díl je montážní sestava, pravděpodobně mimo rozsah, ověřit v TARIC.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>7307990000</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Sestava vyrovnávacího kohoutu zásobníku na prach</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>30600162250</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>284.96</v>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>CBAM</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>CBAM zboží (železo/ocel, kap. 73). Čistá hmotnost pouze 1 kg – hluboko pod limitem de minimis 50 t/rok → kód Y137 v JSD (potvrdit se zákazníkem). Pozor: AD clo na potrubní tvarovky z CN (ex 7307 99 80, 58,6 %) – ověřit v TARIC, zda se na díl vztahuje (pravděpodobně ne, není svařovací tvarovka).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F7" s="5" t="n">
         <v>1506.5</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G7" s="5" t="n">
         <v>2327.5</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>229167.21</v>
       </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9"/>
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Legenda:</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Legenda:</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>🟡 ORANŽOVÁ</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CBAM zboží (železo/ocel) – celkem jen 1,5 kg NW; navrhnout kód Y137 (de minimis) v JSD</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>🟡 ORANŽOVÁ</t>
+          <t>🟨 SVĚTLE ŽLUTÁ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CBAM zboží (železo/ocel) – celkem jen 1,5 kg NW; navrhnout kód Y137 (de minimis) v JSD</t>
+          <t>OVĚŘIT – čínský exportní kód bez přímého EU ekvivalentu, zkontrolovat zařazení v TARIC před podáním JSD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>HS kódy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Vše CN (Čína) – BEZ preferenční věty na fakturách → standardní sazba třetí země (žádná preference EU–CN neexistuje)</t>
+          <t>Kódy na fakturách jsou čínské exportní („Orig Export HS"). Pro JSD platí EU TARIC – 8421392990 + 8421392290 sloučeny pod 8421 39 25 90 (filtrace vzduchu).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Vše CN (Čína) – BEZ preferenční věty na fakturách → standardní sazba třetí země</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Kontrola</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>GW 2327,5 kg a 31 nákladových kusů souhlasí s HBL DK26050913; hodnoty souhlasí se 4 fakturami (celkem 229 167,21 CNY)</t>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>GW 2327,5 kg a 31 kusů souhlasí s HBL DK26050913; hodnota souhlasí se 4 fakturami (229 167,21 CNY)</t>
         </is>
       </c>
     </row>
@@ -823,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -877,7 +897,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="5">
         <f>== PŘIJATÉ DOKUMENTY (stav 10.7.2026) ===</f>
@@ -919,7 +938,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="5">
         <f>== PREFERENČNÍ VĚTA / COO – DŮLEŽITÉ ===</f>
@@ -947,7 +965,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="5">
         <f>== CBAM ===</f>
@@ -975,7 +992,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="5">
         <f>== ANTIDUMPING ===</f>
@@ -1003,7 +1019,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="5">
         <f>== POZNÁMKY / NESROVNALOSTI ===</f>
@@ -1031,6 +1046,47 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="5">
+        <f>== HS KÓDY – ČÍNSKÉ vs. EU (aktualizace) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Kódy na fakturách/master seznamu jsou ČÍNSKÉ exportní kódy („Orig Export HS"), ne EU TARIC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Čínské 8421392990 (sběrače prachu) a 8421392290 (UMA jednotky) v EU nomenklatuře neexistují – EU má pro filtraci vzduchu jediný kód 8421 39 25 (TARIC 8421 39 25 90 – ostatní).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>→ Obě skupiny sloučeny do jednoho řádku 8421392590: 25 ks, NW 1 420 kg, GW 2 160 kg, 216 500,61 CNY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Zbývající kódy k ověření v TARIC: 8421199090 (EU členění 8421 19 je odlišné) a 8421999090 (EU 8421 99 90). 7318230000 má v EU přímý ekvivalent, 7307990000 → EU 7307 99 80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>HBL uvádí HS 842139 – konzistentní s hlavní položkou 8421 39 25 90.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>